<commit_message>
auto: update dengue data 2026-04-05
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,32 +418,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>who_cases_monthly</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>google_trends_dengue_fever</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>google_trends_dengue_vaccine</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>wikipedia_total_dengue_views</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>wikipedia_mosquito_views_total</t>
         </is>
@@ -492,7 +480,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E3" t="n">
         <v>10100</v>
@@ -509,7 +497,7 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
         <v>25</v>
@@ -532,7 +520,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -552,7 +540,7 @@
         <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -572,7 +560,7 @@
         <v>13</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -589,10 +577,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -609,10 +597,10 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D9" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -629,10 +617,10 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D10" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E10" t="n">
         <v>55083</v>
@@ -672,7 +660,7 @@
         <v>57</v>
       </c>
       <c r="D12" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E12" t="n">
         <v>33621</v>
@@ -692,7 +680,7 @@
         <v>24</v>
       </c>
       <c r="D13" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E13" t="n">
         <v>16159</v>
@@ -712,7 +700,7 @@
         <v>23</v>
       </c>
       <c r="D14" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -752,7 +740,7 @@
         <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E16" t="n">
         <v>9603</v>
@@ -772,7 +760,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E17" t="n">
         <v>9781</v>
@@ -809,10 +797,10 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D19" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E19" t="n">
         <v>15980</v>
@@ -829,7 +817,7 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D20" t="n">
         <v>34</v>
@@ -849,10 +837,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D21" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -869,10 +857,10 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D22" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E22" t="n">
         <v>57125</v>
@@ -889,7 +877,7 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D23" t="n">
         <v>54</v>
@@ -909,7 +897,7 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D24" t="n">
         <v>55</v>
@@ -929,10 +917,10 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D25" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -949,7 +937,7 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D26" t="n">
         <v>25</v>
@@ -969,10 +957,10 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D27" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E27" t="n">
         <v>15761</v>
@@ -989,7 +977,7 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D28" t="n">
         <v>29</v>
@@ -1012,7 +1000,7 @@
         <v>14</v>
       </c>
       <c r="D29" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E29" t="n">
         <v>10272</v>
@@ -1032,7 +1020,7 @@
         <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E30" t="n">
         <v>18743</v>
@@ -1052,7 +1040,7 @@
         <v>27</v>
       </c>
       <c r="D31" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E31" t="n">
         <v>29014</v>
@@ -1072,7 +1060,7 @@
         <v>39</v>
       </c>
       <c r="D32" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
@@ -1089,10 +1077,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D33" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1109,10 +1097,10 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D34" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1149,10 +1137,10 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D36" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E36" t="n">
         <v>60939</v>
@@ -1169,10 +1157,10 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D37" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
@@ -1191,7 +1179,7 @@
         <v>5079</v>
       </c>
       <c r="C38" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D38" t="n">
         <v>30</v>
@@ -1235,10 +1223,10 @@
         <v>5597</v>
       </c>
       <c r="C40" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D40" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1260,7 +1248,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1282,7 +1270,7 @@
         <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E42" t="n">
         <v>14543</v>
@@ -1301,7 +1289,7 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D43" t="n">
         <v>36</v>
@@ -1323,10 +1311,10 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D44" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E44" t="n">
         <v>29905</v>
@@ -1345,10 +1333,10 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D45" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1367,10 +1355,10 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D46" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E46" t="n">
         <v>22844</v>
@@ -1392,7 +1380,7 @@
         <v>54</v>
       </c>
       <c r="D47" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
@@ -1414,7 +1402,7 @@
         <v>32</v>
       </c>
       <c r="D48" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1436,7 +1424,7 @@
         <v>17</v>
       </c>
       <c r="D49" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E49" t="n">
         <v>10532</v>
@@ -1458,7 +1446,7 @@
         <v>13</v>
       </c>
       <c r="D50" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E50" t="n">
         <v>9411</v>
@@ -1477,10 +1465,10 @@
         <v>3806</v>
       </c>
       <c r="C51" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D51" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E51" t="n">
         <v>5840</v>
@@ -1502,7 +1490,7 @@
         <v>10</v>
       </c>
       <c r="D52" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E52" t="n">
         <v>5131</v>
@@ -1524,7 +1512,7 @@
         <v>9</v>
       </c>
       <c r="D53" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1568,7 +1556,7 @@
         <v>13</v>
       </c>
       <c r="D55" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
@@ -1590,7 +1578,7 @@
         <v>18</v>
       </c>
       <c r="D56" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1609,10 +1597,10 @@
         <v>14303</v>
       </c>
       <c r="C57" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D57" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1631,7 +1619,7 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D58" t="n">
         <v>36</v>
@@ -1678,7 +1666,7 @@
         <v>17</v>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1697,10 +1685,10 @@
         <v>7539</v>
       </c>
       <c r="C61" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D61" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1744,7 +1732,7 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1764,7 +1752,7 @@
         <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1804,12 +1792,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>open_dengue_national_yearly</t>
         </is>

</xml_diff>

<commit_message>
auto: update dengue data 2026-04-20
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,6 +445,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>wikipedia_total_dengue_views_normalized</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>wikipedia_mosquito_views_total</t>
         </is>
       </c>
@@ -460,12 +465,15 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E2" t="n">
         <v>10782</v>
       </c>
       <c r="F2" t="n">
+        <v>3129.2189</v>
+      </c>
+      <c r="G2" t="n">
         <v>4403</v>
       </c>
     </row>
@@ -486,6 +494,9 @@
         <v>10100</v>
       </c>
       <c r="F3" t="n">
+        <v>2981.6049</v>
+      </c>
+      <c r="G3" t="n">
         <v>5913</v>
       </c>
     </row>
@@ -506,6 +517,9 @@
         <v>10289</v>
       </c>
       <c r="F4" t="n">
+        <v>3208.6276</v>
+      </c>
+      <c r="G4" t="n">
         <v>7598</v>
       </c>
     </row>
@@ -520,12 +534,15 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
       </c>
       <c r="F5" t="n">
+        <v>2849.3583</v>
+      </c>
+      <c r="G5" t="n">
         <v>4811</v>
       </c>
     </row>
@@ -537,15 +554,18 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
       </c>
       <c r="F6" t="n">
+        <v>2184.4783</v>
+      </c>
+      <c r="G6" t="n">
         <v>4792</v>
       </c>
     </row>
@@ -557,15 +577,18 @@
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
       </c>
       <c r="F7" t="n">
+        <v>2911.5361</v>
+      </c>
+      <c r="G7" t="n">
         <v>4905</v>
       </c>
     </row>
@@ -577,15 +600,18 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
       </c>
       <c r="F8" t="n">
+        <v>4433.2881</v>
+      </c>
+      <c r="G8" t="n">
         <v>5539</v>
       </c>
     </row>
@@ -606,6 +632,9 @@
         <v>35620</v>
       </c>
       <c r="F9" t="n">
+        <v>9340.807000000001</v>
+      </c>
+      <c r="G9" t="n">
         <v>5929</v>
       </c>
     </row>
@@ -617,7 +646,7 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D10" t="n">
         <v>79</v>
@@ -626,6 +655,9 @@
         <v>55083</v>
       </c>
       <c r="F10" t="n">
+        <v>18977.9464</v>
+      </c>
+      <c r="G10" t="n">
         <v>6357</v>
       </c>
     </row>
@@ -637,7 +669,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
@@ -646,6 +678,9 @@
         <v>62856</v>
       </c>
       <c r="F11" t="n">
+        <v>25545.1687</v>
+      </c>
+      <c r="G11" t="n">
         <v>7235</v>
       </c>
     </row>
@@ -666,6 +701,9 @@
         <v>33621</v>
       </c>
       <c r="F12" t="n">
+        <v>11923.5522</v>
+      </c>
+      <c r="G12" t="n">
         <v>6668</v>
       </c>
     </row>
@@ -677,15 +715,18 @@
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E13" t="n">
         <v>16159</v>
       </c>
       <c r="F13" t="n">
+        <v>4663.8559</v>
+      </c>
+      <c r="G13" t="n">
         <v>6239</v>
       </c>
     </row>
@@ -697,15 +738,18 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D14" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
       </c>
       <c r="F14" t="n">
+        <v>2851.1882</v>
+      </c>
+      <c r="G14" t="n">
         <v>6117</v>
       </c>
     </row>
@@ -720,12 +764,15 @@
         <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E15" t="n">
         <v>9029</v>
       </c>
       <c r="F15" t="n">
+        <v>2366.7911</v>
+      </c>
+      <c r="G15" t="n">
         <v>4745</v>
       </c>
     </row>
@@ -740,12 +787,15 @@
         <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E16" t="n">
         <v>9603</v>
       </c>
       <c r="F16" t="n">
+        <v>2598.8767</v>
+      </c>
+      <c r="G16" t="n">
         <v>7667</v>
       </c>
     </row>
@@ -766,6 +816,9 @@
         <v>9781</v>
       </c>
       <c r="F17" t="n">
+        <v>2548.3312</v>
+      </c>
+      <c r="G17" t="n">
         <v>6154</v>
       </c>
     </row>
@@ -780,12 +833,15 @@
         <v>14</v>
       </c>
       <c r="D18" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E18" t="n">
         <v>10872</v>
       </c>
       <c r="F18" t="n">
+        <v>1997.5654</v>
+      </c>
+      <c r="G18" t="n">
         <v>5267</v>
       </c>
     </row>
@@ -800,12 +856,15 @@
         <v>18</v>
       </c>
       <c r="D19" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" t="n">
         <v>15980</v>
       </c>
       <c r="F19" t="n">
+        <v>3072.4912</v>
+      </c>
+      <c r="G19" t="n">
         <v>4768</v>
       </c>
     </row>
@@ -820,12 +879,15 @@
         <v>26</v>
       </c>
       <c r="D20" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
       </c>
       <c r="F20" t="n">
+        <v>4101.412</v>
+      </c>
+      <c r="G20" t="n">
         <v>7618</v>
       </c>
     </row>
@@ -840,12 +902,15 @@
         <v>38</v>
       </c>
       <c r="D21" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
       </c>
       <c r="F21" t="n">
+        <v>6089.7509</v>
+      </c>
+      <c r="G21" t="n">
         <v>8494</v>
       </c>
     </row>
@@ -857,7 +922,7 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D22" t="n">
         <v>52</v>
@@ -866,6 +931,9 @@
         <v>57125</v>
       </c>
       <c r="F22" t="n">
+        <v>12615.5129</v>
+      </c>
+      <c r="G22" t="n">
         <v>8979</v>
       </c>
     </row>
@@ -877,7 +945,7 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D23" t="n">
         <v>54</v>
@@ -886,6 +954,9 @@
         <v>76590</v>
       </c>
       <c r="F23" t="n">
+        <v>19115.2163</v>
+      </c>
+      <c r="G23" t="n">
         <v>9480</v>
       </c>
     </row>
@@ -906,6 +977,9 @@
         <v>74792</v>
       </c>
       <c r="F24" t="n">
+        <v>17743.3223</v>
+      </c>
+      <c r="G24" t="n">
         <v>9845</v>
       </c>
     </row>
@@ -917,7 +991,7 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D25" t="n">
         <v>32</v>
@@ -926,6 +1000,9 @@
         <v>20815</v>
       </c>
       <c r="F25" t="n">
+        <v>4299.3351</v>
+      </c>
+      <c r="G25" t="n">
         <v>4974</v>
       </c>
     </row>
@@ -946,6 +1023,9 @@
         <v>14129</v>
       </c>
       <c r="F26" t="n">
+        <v>3051.7552</v>
+      </c>
+      <c r="G26" t="n">
         <v>4798</v>
       </c>
     </row>
@@ -957,15 +1037,18 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E27" t="n">
         <v>15761</v>
       </c>
       <c r="F27" t="n">
+        <v>3130.4701</v>
+      </c>
+      <c r="G27" t="n">
         <v>6885</v>
       </c>
     </row>
@@ -977,7 +1060,7 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D28" t="n">
         <v>29</v>
@@ -986,6 +1069,9 @@
         <v>15308</v>
       </c>
       <c r="F28" t="n">
+        <v>2798.3631</v>
+      </c>
+      <c r="G28" t="n">
         <v>9348</v>
       </c>
     </row>
@@ -997,15 +1083,18 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E29" t="n">
         <v>10272</v>
       </c>
       <c r="F29" t="n">
+        <v>1858.0278</v>
+      </c>
+      <c r="G29" t="n">
         <v>6039</v>
       </c>
     </row>
@@ -1026,6 +1115,9 @@
         <v>18743</v>
       </c>
       <c r="F30" t="n">
+        <v>3090.554</v>
+      </c>
+      <c r="G30" t="n">
         <v>6711</v>
       </c>
     </row>
@@ -1037,15 +1129,18 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D31" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E31" t="n">
         <v>29014</v>
       </c>
       <c r="F31" t="n">
+        <v>3310.0027</v>
+      </c>
+      <c r="G31" t="n">
         <v>5541</v>
       </c>
     </row>
@@ -1060,12 +1155,15 @@
         <v>39</v>
       </c>
       <c r="D32" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
       </c>
       <c r="F32" t="n">
+        <v>8340.5954</v>
+      </c>
+      <c r="G32" t="n">
         <v>8574</v>
       </c>
     </row>
@@ -1077,15 +1175,18 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
       </c>
       <c r="F33" t="n">
+        <v>11603.5597</v>
+      </c>
+      <c r="G33" t="n">
         <v>9101</v>
       </c>
     </row>
@@ -1097,15 +1198,18 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D34" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
       </c>
       <c r="F34" t="n">
+        <v>19082.9673</v>
+      </c>
+      <c r="G34" t="n">
         <v>7299</v>
       </c>
     </row>
@@ -1120,12 +1224,15 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
       </c>
       <c r="F35" t="n">
+        <v>13542.0717</v>
+      </c>
+      <c r="G35" t="n">
         <v>8011</v>
       </c>
     </row>
@@ -1137,15 +1244,18 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D36" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E36" t="n">
         <v>60939</v>
       </c>
       <c r="F36" t="n">
+        <v>8275.5723</v>
+      </c>
+      <c r="G36" t="n">
         <v>7745</v>
       </c>
     </row>
@@ -1157,15 +1267,18 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D37" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
       </c>
       <c r="F37" t="n">
+        <v>3525.8816</v>
+      </c>
+      <c r="G37" t="n">
         <v>7888</v>
       </c>
     </row>
@@ -1179,15 +1292,18 @@
         <v>5079</v>
       </c>
       <c r="C38" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D38" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E38" t="n">
         <v>17390</v>
       </c>
       <c r="F38" t="n">
+        <v>2407.4712</v>
+      </c>
+      <c r="G38" t="n">
         <v>5887</v>
       </c>
     </row>
@@ -1210,6 +1326,9 @@
         <v>15334</v>
       </c>
       <c r="F39" t="n">
+        <v>2340.3037</v>
+      </c>
+      <c r="G39" t="n">
         <v>8059</v>
       </c>
     </row>
@@ -1223,15 +1342,18 @@
         <v>5597</v>
       </c>
       <c r="C40" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D40" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
       </c>
       <c r="F40" t="n">
+        <v>1849.6489</v>
+      </c>
+      <c r="G40" t="n">
         <v>7211</v>
       </c>
     </row>
@@ -1254,6 +1376,9 @@
         <v>10261</v>
       </c>
       <c r="F41" t="n">
+        <v>1364.129</v>
+      </c>
+      <c r="G41" t="n">
         <v>5874</v>
       </c>
     </row>
@@ -1276,6 +1401,9 @@
         <v>14543</v>
       </c>
       <c r="F42" t="n">
+        <v>1592.341</v>
+      </c>
+      <c r="G42" t="n">
         <v>3498</v>
       </c>
     </row>
@@ -1289,7 +1417,7 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D43" t="n">
         <v>36</v>
@@ -1298,6 +1426,9 @@
         <v>16505</v>
       </c>
       <c r="F43" t="n">
+        <v>1555.0182</v>
+      </c>
+      <c r="G43" t="n">
         <v>2875</v>
       </c>
     </row>
@@ -1311,15 +1442,18 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D44" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E44" t="n">
         <v>29905</v>
       </c>
       <c r="F44" t="n">
+        <v>2828.7245</v>
+      </c>
+      <c r="G44" t="n">
         <v>4652</v>
       </c>
     </row>
@@ -1333,15 +1467,18 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D45" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
       </c>
       <c r="F45" t="n">
+        <v>2100.1749</v>
+      </c>
+      <c r="G45" t="n">
         <v>4483</v>
       </c>
     </row>
@@ -1355,7 +1492,7 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D46" t="n">
         <v>55</v>
@@ -1364,6 +1501,9 @@
         <v>22844</v>
       </c>
       <c r="F46" t="n">
+        <v>2551.7948</v>
+      </c>
+      <c r="G46" t="n">
         <v>3434</v>
       </c>
     </row>
@@ -1377,15 +1517,18 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D47" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
       </c>
       <c r="F47" t="n">
+        <v>2677.8742</v>
+      </c>
+      <c r="G47" t="n">
         <v>3449</v>
       </c>
     </row>
@@ -1399,15 +1542,18 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D48" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
       </c>
       <c r="F48" t="n">
+        <v>2133.5331</v>
+      </c>
+      <c r="G48" t="n">
         <v>2863</v>
       </c>
     </row>
@@ -1424,12 +1570,15 @@
         <v>17</v>
       </c>
       <c r="D49" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E49" t="n">
         <v>10532</v>
       </c>
       <c r="F49" t="n">
+        <v>1169.4372</v>
+      </c>
+      <c r="G49" t="n">
         <v>2420</v>
       </c>
     </row>
@@ -1443,15 +1592,18 @@
         <v>4700</v>
       </c>
       <c r="C50" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D50" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E50" t="n">
         <v>9411</v>
       </c>
       <c r="F50" t="n">
+        <v>1067.1823</v>
+      </c>
+      <c r="G50" t="n">
         <v>2276</v>
       </c>
     </row>
@@ -1468,12 +1620,15 @@
         <v>10</v>
       </c>
       <c r="D51" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E51" t="n">
         <v>5840</v>
       </c>
       <c r="F51" t="n">
+        <v>742.0104</v>
+      </c>
+      <c r="G51" t="n">
         <v>2259</v>
       </c>
     </row>
@@ -1490,12 +1645,15 @@
         <v>10</v>
       </c>
       <c r="D52" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E52" t="n">
         <v>5131</v>
       </c>
       <c r="F52" t="n">
+        <v>655.7098</v>
+      </c>
+      <c r="G52" t="n">
         <v>2625</v>
       </c>
     </row>
@@ -1509,15 +1667,18 @@
         <v>2700</v>
       </c>
       <c r="C53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
       </c>
       <c r="F53" t="n">
+        <v>602.5579</v>
+      </c>
+      <c r="G53" t="n">
         <v>2018</v>
       </c>
     </row>
@@ -1540,6 +1701,9 @@
         <v>7995</v>
       </c>
       <c r="F54" t="n">
+        <v>792.1904</v>
+      </c>
+      <c r="G54" t="n">
         <v>2166</v>
       </c>
     </row>
@@ -1556,12 +1720,15 @@
         <v>13</v>
       </c>
       <c r="D55" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
       </c>
       <c r="F55" t="n">
+        <v>791.9278</v>
+      </c>
+      <c r="G55" t="n">
         <v>2900</v>
       </c>
     </row>
@@ -1578,12 +1745,15 @@
         <v>18</v>
       </c>
       <c r="D56" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
       </c>
       <c r="F56" t="n">
+        <v>852.0587</v>
+      </c>
+      <c r="G56" t="n">
         <v>2166</v>
       </c>
     </row>
@@ -1597,15 +1767,18 @@
         <v>14303</v>
       </c>
       <c r="C57" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D57" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
       </c>
       <c r="F57" t="n">
+        <v>1100.9271</v>
+      </c>
+      <c r="G57" t="n">
         <v>3055</v>
       </c>
     </row>
@@ -1619,15 +1792,18 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D58" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E58" t="n">
         <v>7044</v>
       </c>
       <c r="F58" t="n">
+        <v>908.633</v>
+      </c>
+      <c r="G58" t="n">
         <v>3025</v>
       </c>
     </row>
@@ -1644,12 +1820,15 @@
         <v>20</v>
       </c>
       <c r="D59" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E59" t="n">
         <v>6021</v>
       </c>
       <c r="F59" t="n">
+        <v>771.3006</v>
+      </c>
+      <c r="G59" t="n">
         <v>2743</v>
       </c>
     </row>
@@ -1672,6 +1851,9 @@
         <v>5358</v>
       </c>
       <c r="F60" t="n">
+        <v>668.6939</v>
+      </c>
+      <c r="G60" t="n">
         <v>2282</v>
       </c>
     </row>
@@ -1694,6 +1876,9 @@
         <v>3621</v>
       </c>
       <c r="F61" t="n">
+        <v>488.4914</v>
+      </c>
+      <c r="G61" t="n">
         <v>2029</v>
       </c>
     </row>
@@ -1716,6 +1901,9 @@
         <v>2259</v>
       </c>
       <c r="F62" t="n">
+        <v>291.1217</v>
+      </c>
+      <c r="G62" t="n">
         <v>1846</v>
       </c>
     </row>
@@ -1732,12 +1920,15 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
       </c>
       <c r="F63" t="n">
+        <v>279.3269</v>
+      </c>
+      <c r="G63" t="n">
         <v>1978</v>
       </c>
     </row>
@@ -1752,12 +1943,15 @@
         <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
       </c>
       <c r="F64" t="n">
+        <v>358.422</v>
+      </c>
+      <c r="G64" t="n">
         <v>3686</v>
       </c>
     </row>
@@ -1774,6 +1968,9 @@
         <v>69</v>
       </c>
       <c r="F65" t="n">
+        <v>9.833399999999999</v>
+      </c>
+      <c r="G65" t="n">
         <v>114</v>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: update dengue data 2026-05-05
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,7 +474,7 @@
         <v>3129.2189</v>
       </c>
       <c r="G2" t="n">
-        <v>4403</v>
+        <v>4016</v>
       </c>
     </row>
     <row r="3">
@@ -497,7 +497,7 @@
         <v>2981.6049</v>
       </c>
       <c r="G3" t="n">
-        <v>5913</v>
+        <v>5137</v>
       </c>
     </row>
     <row r="4">
@@ -511,7 +511,7 @@
         <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" t="n">
         <v>10289</v>
@@ -520,7 +520,7 @@
         <v>3208.6276</v>
       </c>
       <c r="G4" t="n">
-        <v>7598</v>
+        <v>6699</v>
       </c>
     </row>
     <row r="5">
@@ -534,7 +534,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -543,7 +543,7 @@
         <v>2849.3583</v>
       </c>
       <c r="G5" t="n">
-        <v>4811</v>
+        <v>4463</v>
       </c>
     </row>
     <row r="6">
@@ -557,7 +557,7 @@
         <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -566,7 +566,7 @@
         <v>2184.4783</v>
       </c>
       <c r="G6" t="n">
-        <v>4792</v>
+        <v>4546</v>
       </c>
     </row>
     <row r="7">
@@ -580,7 +580,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -589,7 +589,7 @@
         <v>2911.5361</v>
       </c>
       <c r="G7" t="n">
-        <v>4905</v>
+        <v>4369</v>
       </c>
     </row>
     <row r="8">
@@ -600,10 +600,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D8" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -612,7 +612,7 @@
         <v>4433.2881</v>
       </c>
       <c r="G8" t="n">
-        <v>5539</v>
+        <v>5056</v>
       </c>
     </row>
     <row r="9">
@@ -635,7 +635,7 @@
         <v>9340.807000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>5929</v>
+        <v>5463</v>
       </c>
     </row>
     <row r="10">
@@ -646,7 +646,7 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D10" t="n">
         <v>79</v>
@@ -658,7 +658,7 @@
         <v>18977.9464</v>
       </c>
       <c r="G10" t="n">
-        <v>6357</v>
+        <v>5855</v>
       </c>
     </row>
     <row r="11">
@@ -681,7 +681,7 @@
         <v>25545.1687</v>
       </c>
       <c r="G11" t="n">
-        <v>7235</v>
+        <v>6830</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +692,7 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" t="n">
         <v>62</v>
@@ -704,7 +704,7 @@
         <v>11923.5522</v>
       </c>
       <c r="G12" t="n">
-        <v>6668</v>
+        <v>6229</v>
       </c>
     </row>
     <row r="13">
@@ -718,7 +718,7 @@
         <v>25</v>
       </c>
       <c r="D13" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" t="n">
         <v>16159</v>
@@ -727,7 +727,7 @@
         <v>4663.8559</v>
       </c>
       <c r="G13" t="n">
-        <v>6239</v>
+        <v>5617</v>
       </c>
     </row>
     <row r="14">
@@ -738,10 +738,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D14" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -750,7 +750,7 @@
         <v>2851.1882</v>
       </c>
       <c r="G14" t="n">
-        <v>6117</v>
+        <v>5713</v>
       </c>
     </row>
     <row r="15">
@@ -773,7 +773,7 @@
         <v>2366.7911</v>
       </c>
       <c r="G15" t="n">
-        <v>4745</v>
+        <v>4335</v>
       </c>
     </row>
     <row r="16">
@@ -796,7 +796,7 @@
         <v>2598.8767</v>
       </c>
       <c r="G16" t="n">
-        <v>7667</v>
+        <v>7246</v>
       </c>
     </row>
     <row r="17">
@@ -819,7 +819,7 @@
         <v>2548.3312</v>
       </c>
       <c r="G17" t="n">
-        <v>6154</v>
+        <v>5613</v>
       </c>
     </row>
     <row r="18">
@@ -833,7 +833,7 @@
         <v>14</v>
       </c>
       <c r="D18" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E18" t="n">
         <v>10872</v>
@@ -842,7 +842,7 @@
         <v>1997.5654</v>
       </c>
       <c r="G18" t="n">
-        <v>5267</v>
+        <v>4745</v>
       </c>
     </row>
     <row r="19">
@@ -853,10 +853,10 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D19" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E19" t="n">
         <v>15980</v>
@@ -865,7 +865,7 @@
         <v>3072.4912</v>
       </c>
       <c r="G19" t="n">
-        <v>4768</v>
+        <v>4053</v>
       </c>
     </row>
     <row r="20">
@@ -888,7 +888,7 @@
         <v>4101.412</v>
       </c>
       <c r="G20" t="n">
-        <v>7618</v>
+        <v>6549</v>
       </c>
     </row>
     <row r="21">
@@ -899,7 +899,7 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D21" t="n">
         <v>35</v>
@@ -911,7 +911,7 @@
         <v>6089.7509</v>
       </c>
       <c r="G21" t="n">
-        <v>8494</v>
+        <v>7663</v>
       </c>
     </row>
     <row r="22">
@@ -934,7 +934,7 @@
         <v>12615.5129</v>
       </c>
       <c r="G22" t="n">
-        <v>8979</v>
+        <v>8289</v>
       </c>
     </row>
     <row r="23">
@@ -945,10 +945,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D23" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -957,7 +957,7 @@
         <v>19115.2163</v>
       </c>
       <c r="G23" t="n">
-        <v>9480</v>
+        <v>8785</v>
       </c>
     </row>
     <row r="24">
@@ -968,10 +968,10 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D24" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E24" t="n">
         <v>74792</v>
@@ -980,7 +980,7 @@
         <v>17743.3223</v>
       </c>
       <c r="G24" t="n">
-        <v>9845</v>
+        <v>9289</v>
       </c>
     </row>
     <row r="25">
@@ -994,7 +994,7 @@
         <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -1003,7 +1003,7 @@
         <v>4299.3351</v>
       </c>
       <c r="G25" t="n">
-        <v>4974</v>
+        <v>4520</v>
       </c>
     </row>
     <row r="26">
@@ -1026,7 +1026,7 @@
         <v>3051.7552</v>
       </c>
       <c r="G26" t="n">
-        <v>4798</v>
+        <v>4432</v>
       </c>
     </row>
     <row r="27">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D27" t="n">
         <v>33</v>
@@ -1049,7 +1049,7 @@
         <v>3130.4701</v>
       </c>
       <c r="G27" t="n">
-        <v>6885</v>
+        <v>6233</v>
       </c>
     </row>
     <row r="28">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D28" t="n">
         <v>29</v>
@@ -1072,7 +1072,7 @@
         <v>2798.3631</v>
       </c>
       <c r="G28" t="n">
-        <v>9348</v>
+        <v>8913</v>
       </c>
     </row>
     <row r="29">
@@ -1095,7 +1095,7 @@
         <v>1858.0278</v>
       </c>
       <c r="G29" t="n">
-        <v>6039</v>
+        <v>5732</v>
       </c>
     </row>
     <row r="30">
@@ -1118,7 +1118,7 @@
         <v>3090.554</v>
       </c>
       <c r="G30" t="n">
-        <v>6711</v>
+        <v>6207</v>
       </c>
     </row>
     <row r="31">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D31" t="n">
         <v>30</v>
@@ -1141,7 +1141,7 @@
         <v>3310.0027</v>
       </c>
       <c r="G31" t="n">
-        <v>5541</v>
+        <v>5063</v>
       </c>
     </row>
     <row r="32">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D32" t="n">
         <v>37</v>
@@ -1164,7 +1164,7 @@
         <v>8340.5954</v>
       </c>
       <c r="G32" t="n">
-        <v>8574</v>
+        <v>7516</v>
       </c>
     </row>
     <row r="33">
@@ -1178,7 +1178,7 @@
         <v>68</v>
       </c>
       <c r="D33" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1187,7 +1187,7 @@
         <v>11603.5597</v>
       </c>
       <c r="G33" t="n">
-        <v>9101</v>
+        <v>7698</v>
       </c>
     </row>
     <row r="34">
@@ -1198,10 +1198,10 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D34" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1210,7 +1210,7 @@
         <v>19082.9673</v>
       </c>
       <c r="G34" t="n">
-        <v>7299</v>
+        <v>6717</v>
       </c>
     </row>
     <row r="35">
@@ -1224,7 +1224,7 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1233,7 +1233,7 @@
         <v>13542.0717</v>
       </c>
       <c r="G35" t="n">
-        <v>8011</v>
+        <v>7616</v>
       </c>
     </row>
     <row r="36">
@@ -1244,10 +1244,10 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D36" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E36" t="n">
         <v>60939</v>
@@ -1256,7 +1256,7 @@
         <v>8275.5723</v>
       </c>
       <c r="G36" t="n">
-        <v>7745</v>
+        <v>7099</v>
       </c>
     </row>
     <row r="37">
@@ -1267,10 +1267,10 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D37" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
@@ -1279,7 +1279,7 @@
         <v>3525.8816</v>
       </c>
       <c r="G37" t="n">
-        <v>7888</v>
+        <v>7273</v>
       </c>
     </row>
     <row r="38">
@@ -1304,7 +1304,7 @@
         <v>2407.4712</v>
       </c>
       <c r="G38" t="n">
-        <v>5887</v>
+        <v>5346</v>
       </c>
     </row>
     <row r="39">
@@ -1329,7 +1329,7 @@
         <v>2340.3037</v>
       </c>
       <c r="G39" t="n">
-        <v>8059</v>
+        <v>7445</v>
       </c>
     </row>
     <row r="40">
@@ -1345,7 +1345,7 @@
         <v>13</v>
       </c>
       <c r="D40" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1354,7 +1354,7 @@
         <v>1849.6489</v>
       </c>
       <c r="G40" t="n">
-        <v>7211</v>
+        <v>6714</v>
       </c>
     </row>
     <row r="41">
@@ -1379,7 +1379,7 @@
         <v>1364.129</v>
       </c>
       <c r="G41" t="n">
-        <v>5874</v>
+        <v>5552</v>
       </c>
     </row>
     <row r="42">
@@ -1395,7 +1395,7 @@
         <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E42" t="n">
         <v>14543</v>
@@ -1404,7 +1404,7 @@
         <v>1592.341</v>
       </c>
       <c r="G42" t="n">
-        <v>3498</v>
+        <v>3082</v>
       </c>
     </row>
     <row r="43">
@@ -1417,7 +1417,7 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D43" t="n">
         <v>36</v>
@@ -1429,7 +1429,7 @@
         <v>1555.0182</v>
       </c>
       <c r="G43" t="n">
-        <v>2875</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="44">
@@ -1442,7 +1442,7 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D44" t="n">
         <v>62</v>
@@ -1454,7 +1454,7 @@
         <v>2828.7245</v>
       </c>
       <c r="G44" t="n">
-        <v>4652</v>
+        <v>3467</v>
       </c>
     </row>
     <row r="45">
@@ -1467,10 +1467,10 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D45" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1479,7 +1479,7 @@
         <v>2100.1749</v>
       </c>
       <c r="G45" t="n">
-        <v>4483</v>
+        <v>3928</v>
       </c>
     </row>
     <row r="46">
@@ -1492,7 +1492,7 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D46" t="n">
         <v>55</v>
@@ -1504,7 +1504,7 @@
         <v>2551.7948</v>
       </c>
       <c r="G46" t="n">
-        <v>3434</v>
+        <v>3018</v>
       </c>
     </row>
     <row r="47">
@@ -1517,10 +1517,10 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D47" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
@@ -1529,7 +1529,7 @@
         <v>2677.8742</v>
       </c>
       <c r="G47" t="n">
-        <v>3449</v>
+        <v>3071</v>
       </c>
     </row>
     <row r="48">
@@ -1542,7 +1542,7 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D48" t="n">
         <v>47</v>
@@ -1554,7 +1554,7 @@
         <v>2133.5331</v>
       </c>
       <c r="G48" t="n">
-        <v>2863</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="49">
@@ -1579,7 +1579,7 @@
         <v>1169.4372</v>
       </c>
       <c r="G49" t="n">
-        <v>2420</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="50">
@@ -1604,7 +1604,7 @@
         <v>1067.1823</v>
       </c>
       <c r="G50" t="n">
-        <v>2276</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="51">
@@ -1620,7 +1620,7 @@
         <v>10</v>
       </c>
       <c r="D51" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E51" t="n">
         <v>5840</v>
@@ -1629,7 +1629,7 @@
         <v>742.0104</v>
       </c>
       <c r="G51" t="n">
-        <v>2259</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="52">
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="D52" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E52" t="n">
         <v>5131</v>
@@ -1654,7 +1654,7 @@
         <v>655.7098</v>
       </c>
       <c r="G52" t="n">
-        <v>2625</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="53">
@@ -1670,7 +1670,7 @@
         <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1679,7 +1679,7 @@
         <v>602.5579</v>
       </c>
       <c r="G53" t="n">
-        <v>2018</v>
+        <v>1769</v>
       </c>
     </row>
     <row r="54">
@@ -1704,7 +1704,7 @@
         <v>792.1904</v>
       </c>
       <c r="G54" t="n">
-        <v>2166</v>
+        <v>1765</v>
       </c>
     </row>
     <row r="55">
@@ -1720,7 +1720,7 @@
         <v>13</v>
       </c>
       <c r="D55" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
@@ -1729,7 +1729,7 @@
         <v>791.9278</v>
       </c>
       <c r="G55" t="n">
-        <v>2900</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="56">
@@ -1754,7 +1754,7 @@
         <v>852.0587</v>
       </c>
       <c r="G56" t="n">
-        <v>2166</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="57">
@@ -1767,10 +1767,10 @@
         <v>14303</v>
       </c>
       <c r="C57" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D57" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1779,7 +1779,7 @@
         <v>1100.9271</v>
       </c>
       <c r="G57" t="n">
-        <v>3055</v>
+        <v>2709</v>
       </c>
     </row>
     <row r="58">
@@ -1792,10 +1792,10 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E58" t="n">
         <v>7044</v>
@@ -1804,7 +1804,7 @@
         <v>908.633</v>
       </c>
       <c r="G58" t="n">
-        <v>3025</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="59">
@@ -1820,7 +1820,7 @@
         <v>20</v>
       </c>
       <c r="D59" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E59" t="n">
         <v>6021</v>
@@ -1829,7 +1829,7 @@
         <v>771.3006</v>
       </c>
       <c r="G59" t="n">
-        <v>2743</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="60">
@@ -1845,7 +1845,7 @@
         <v>17</v>
       </c>
       <c r="D60" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1854,7 +1854,7 @@
         <v>668.6939</v>
       </c>
       <c r="G60" t="n">
-        <v>2282</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="61">
@@ -1867,10 +1867,10 @@
         <v>7539</v>
       </c>
       <c r="C61" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D61" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1879,7 +1879,7 @@
         <v>488.4914</v>
       </c>
       <c r="G61" t="n">
-        <v>2029</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="62">
@@ -1895,7 +1895,7 @@
         <v>8</v>
       </c>
       <c r="D62" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E62" t="n">
         <v>2259</v>
@@ -1904,7 +1904,7 @@
         <v>291.1217</v>
       </c>
       <c r="G62" t="n">
-        <v>1846</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="63">
@@ -1920,7 +1920,7 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1929,7 +1929,7 @@
         <v>279.3269</v>
       </c>
       <c r="G63" t="n">
-        <v>1978</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="64">
@@ -1938,7 +1938,9 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
+      <c r="B64" t="n">
+        <v>3085</v>
+      </c>
       <c r="C64" t="n">
         <v>7</v>
       </c>
@@ -1952,7 +1954,7 @@
         <v>358.422</v>
       </c>
       <c r="G64" t="n">
-        <v>3686</v>
+        <v>3485</v>
       </c>
     </row>
     <row r="65">
@@ -1962,16 +1964,37 @@
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
+      <c r="C65" t="n">
+        <v>6</v>
+      </c>
+      <c r="D65" t="n">
+        <v>38</v>
+      </c>
       <c r="E65" t="n">
-        <v>69</v>
+        <v>2432</v>
       </c>
       <c r="F65" t="n">
         <v>9.833399999999999</v>
       </c>
       <c r="G65" t="n">
-        <v>114</v>
+        <v>3708</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>56</v>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="n">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>